<commit_message>
Add 23 Mar 2026 costing output from BigMint report
Extracted 11 prices from BigMint Daily Report (23 Mar 2026):
- Raipur: P-DRI 26300, Pig Iron 37300, Scrap 34900, SiMn 74.6/kg,
  Iron Ore DRI 30200, Billet 41550, TMT 46200
- NCR: Scrap 35500(-500), Billet 44300(-500), TMT 50600

Margins: Raipur Billet 558.24, TMT 2500.31
         NCR Billet -47.79, TMT 4021.43

Change log now has both 23 Mar and 26 Mar columns.

https://claude.ai/code/session_0134QcDJAg7cq3Eyj1JQx4hr
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -46,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,6 +183,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -544,12 +553,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +575,12 @@
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -577,6 +594,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -592,6 +619,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D3" s="7" t="n">
+        <v>26300</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -607,6 +642,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D4" s="9" t="n">
+        <v>37300</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -620,6 +663,12 @@
       <c r="C5" s="7" t="n">
         <v>34500</v>
       </c>
+      <c r="D5" s="7" t="n">
+        <v>34900</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>35000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -635,6 +684,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D6" s="9" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -650,6 +707,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D7" s="7" t="n">
+        <v>30200</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -667,6 +732,16 @@
           <t>2026-03-26</t>
         </is>
       </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -680,6 +755,12 @@
       <c r="C9" s="13" t="n">
         <v>43250</v>
       </c>
+      <c r="D9" s="13" t="n">
+        <v>41550</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>43800</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -693,6 +774,12 @@
       <c r="C10" s="15" t="n">
         <v>65.27</v>
       </c>
+      <c r="D10" s="15" t="n">
+        <v>558.24</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>-47.79</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -706,6 +793,12 @@
       <c r="C11" s="13" t="n">
         <v>49500</v>
       </c>
+      <c r="D11" s="13" t="n">
+        <v>46200</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>50600</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -718,6 +811,12 @@
       </c>
       <c r="C12" s="15" t="n">
         <v>3589.8</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>2500.31</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>4021.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-10-31
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -46,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -99,12 +99,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -140,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,9 +177,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -553,14 +544,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,16 +560,10 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2025-10-31</t>
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -594,16 +577,6 @@
           <t>NCR</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Raipur</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>NCR</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -612,17 +585,9 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>26300</v>
+        <v>22800</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>25450</v>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -635,17 +600,9 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>37300</v>
+        <v>31800</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="n">
-        <v>37250</v>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -658,16 +615,10 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>34900</v>
+        <v>30200</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>35000</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>34400</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>34500</v>
+        <v>29900</v>
       </c>
     </row>
     <row r="6">
@@ -677,17 +628,9 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>74.59999999999999</v>
+        <v>72</v>
       </c>
       <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -700,17 +643,9 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>30200</v>
+        <v>26800</v>
       </c>
       <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>29500</v>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -724,22 +659,12 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2025-10-31</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
+          <t>2025-10-31</t>
         </is>
       </c>
     </row>
@@ -750,16 +675,10 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>41550</v>
+        <v>34950</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>43800</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>40400</v>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>43250</v>
+        <v>37900</v>
       </c>
     </row>
     <row r="10">
@@ -769,16 +688,10 @@
         </is>
       </c>
       <c r="B10" s="15" t="n">
-        <v>558.24</v>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>-47.79</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>259.94</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>65.27</v>
+        <v>-1433.88</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>-869.46</v>
       </c>
     </row>
     <row r="11">
@@ -788,16 +701,10 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>46200</v>
+        <v>37500</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>50600</v>
-      </c>
-      <c r="D11" s="13" t="n">
-        <v>45200</v>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>49500</v>
+        <v>40600</v>
       </c>
     </row>
     <row r="12">
@@ -807,16 +714,10 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>2500.31</v>
+        <v>-1554.96</v>
       </c>
       <c r="C12" s="15" t="n">
-        <v>4021.43</v>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>2358.82</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>3589.8</v>
+        <v>-859.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-11-29
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -544,12 +544,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +566,12 @@
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -577,6 +585,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -592,6 +610,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D3" s="7" t="n">
+        <v>23750</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -607,6 +633,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D4" s="9" t="n">
+        <v>32400</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -620,6 +654,12 @@
       <c r="C5" s="7" t="n">
         <v>29900</v>
       </c>
+      <c r="D5" s="7" t="n">
+        <v>31000</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>31800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -635,6 +675,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D6" s="9" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -650,6 +698,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D7" s="7" t="n">
+        <v>26950</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -667,6 +723,16 @@
           <t>2025-10-31</t>
         </is>
       </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -680,6 +746,12 @@
       <c r="C9" s="13" t="n">
         <v>37900</v>
       </c>
+      <c r="D9" s="13" t="n">
+        <v>36150</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>39650</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -693,6 +765,12 @@
       <c r="C10" s="15" t="n">
         <v>-869.46</v>
       </c>
+      <c r="D10" s="15" t="n">
+        <v>-1189.77</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>-613.2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -706,6 +784,12 @@
       <c r="C11" s="13" t="n">
         <v>40600</v>
       </c>
+      <c r="D11" s="13" t="n">
+        <v>38900</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>42400</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -718,6 +802,12 @@
       </c>
       <c r="C12" s="15" t="n">
         <v>-859.62</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>-1118.49</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>-565.3099999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-12-20
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -46,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
         <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,6 +183,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -544,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,6 +561,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,6 +583,12 @@
         </is>
       </c>
       <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -595,6 +612,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -618,6 +645,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F3" s="7" t="n">
+        <v>22900</v>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -641,6 +676,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F4" s="9" t="n">
+        <v>33000</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -660,6 +703,12 @@
       <c r="E5" s="7" t="n">
         <v>31800</v>
       </c>
+      <c r="F5" s="7" t="n">
+        <v>31500</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>31700</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -683,6 +732,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F6" s="9" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -706,6 +763,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F7" s="7" t="n">
+        <v>26900</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -733,6 +798,16 @@
           <t>2025-11-29</t>
         </is>
       </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -752,6 +827,12 @@
       <c r="E9" s="13" t="n">
         <v>39650</v>
       </c>
+      <c r="F9" s="13" t="n">
+        <v>37350</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>39800</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -771,6 +852,12 @@
       <c r="E10" s="15" t="n">
         <v>-613.2</v>
       </c>
+      <c r="F10" s="16" t="n">
+        <v>618.4</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>-70.45999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -790,6 +877,12 @@
       <c r="E11" s="13" t="n">
         <v>42400</v>
       </c>
+      <c r="F11" s="13" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>43200</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -808,6 +901,12 @@
       </c>
       <c r="E12" s="15" t="n">
         <v>-565.3099999999999</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>594.55</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>630.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-01-15
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,6 +591,12 @@
         </is>
       </c>
       <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -622,6 +630,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -653,6 +671,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H3" s="7" t="n">
+        <v>24300</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -684,6 +710,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H4" s="9" t="n">
+        <v>37000</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -709,6 +743,12 @@
       <c r="G5" s="7" t="n">
         <v>31700</v>
       </c>
+      <c r="H5" s="7" t="n">
+        <v>33450</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>33600</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -740,6 +780,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H6" s="9" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -771,6 +819,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H7" s="7" t="n">
+        <v>28100</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -808,6 +864,16 @@
           <t>2025-12-20</t>
         </is>
       </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -833,6 +899,12 @@
       <c r="G9" s="13" t="n">
         <v>39800</v>
       </c>
+      <c r="H9" s="13" t="n">
+        <v>40450</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>42400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -858,6 +930,12 @@
       <c r="G10" s="15" t="n">
         <v>-70.45999999999999</v>
       </c>
+      <c r="H10" s="16" t="n">
+        <v>1639.58</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>323.7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -883,6 +961,12 @@
       <c r="G11" s="13" t="n">
         <v>43200</v>
       </c>
+      <c r="H11" s="13" t="n">
+        <v>43500</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>46900</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -907,6 +991,12 @@
       </c>
       <c r="G12" s="16" t="n">
         <v>630.58</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>1999.1</v>
+      </c>
+      <c r="I12" s="16" t="n">
+        <v>2107.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-01-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -565,6 +565,8 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,6 +599,12 @@
         </is>
       </c>
       <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -640,6 +648,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -679,6 +697,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J3" s="7" t="n">
+        <v>25650</v>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -718,6 +744,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J4" s="9" t="n">
+        <v>38000</v>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -749,6 +783,12 @@
       <c r="I5" s="7" t="n">
         <v>33600</v>
       </c>
+      <c r="J5" s="7" t="n">
+        <v>33750</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>34600</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -788,6 +828,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J6" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -827,6 +875,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J7" s="7" t="n">
+        <v>29250</v>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -874,6 +930,16 @@
           <t>2026-01-15</t>
         </is>
       </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -905,6 +971,12 @@
       <c r="I9" s="13" t="n">
         <v>42400</v>
       </c>
+      <c r="J9" s="13" t="n">
+        <v>40950</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>44200</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -936,6 +1008,12 @@
       <c r="I10" s="16" t="n">
         <v>323.7</v>
       </c>
+      <c r="J10" s="16" t="n">
+        <v>676.67</v>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>806.24</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -967,6 +1045,12 @@
       <c r="I11" s="13" t="n">
         <v>46900</v>
       </c>
+      <c r="J11" s="13" t="n">
+        <v>44000</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>48500</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -997,6 +1081,12 @@
       </c>
       <c r="I12" s="16" t="n">
         <v>2107.09</v>
+      </c>
+      <c r="J12" s="16" t="n">
+        <v>1024.48</v>
+      </c>
+      <c r="K12" s="16" t="n">
+        <v>2379.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-02-13
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,6 +567,8 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +607,12 @@
         </is>
       </c>
       <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -658,6 +666,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -705,6 +723,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L3" s="7" t="n">
+        <v>27500</v>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -752,6 +778,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L4" s="9" t="n">
+        <v>38300</v>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -789,6 +823,12 @@
       <c r="K5" s="7" t="n">
         <v>34600</v>
       </c>
+      <c r="L5" s="7" t="n">
+        <v>34850</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>34900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -836,6 +876,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L6" s="9" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -883,6 +931,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L7" s="7" t="n">
+        <v>30450</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -940,6 +996,16 @@
           <t>2026-01-30</t>
         </is>
       </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -977,6 +1043,12 @@
       <c r="K9" s="13" t="n">
         <v>44200</v>
       </c>
+      <c r="L9" s="13" t="n">
+        <v>41550</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>44250</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1014,6 +1086,12 @@
       <c r="K10" s="16" t="n">
         <v>806.24</v>
       </c>
+      <c r="L10" s="15" t="n">
+        <v>-609.77</v>
+      </c>
+      <c r="M10" s="15" t="n">
+        <v>-246.38</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1051,6 +1129,12 @@
       <c r="K11" s="13" t="n">
         <v>48500</v>
       </c>
+      <c r="L11" s="13" t="n">
+        <v>45200</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>48800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1087,6 +1171,12 @@
       </c>
       <c r="K12" s="16" t="n">
         <v>2379.09</v>
+      </c>
+      <c r="L12" s="16" t="n">
+        <v>322.95</v>
+      </c>
+      <c r="M12" s="16" t="n">
+        <v>1567.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-02-27
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -569,6 +569,8 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -613,6 +615,12 @@
         </is>
       </c>
       <c r="M1" s="3" t="n"/>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -676,6 +684,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -731,6 +749,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N3" s="7" t="n">
+        <v>26100</v>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -786,6 +812,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N4" s="9" t="n">
+        <v>37950</v>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -829,6 +863,12 @@
       <c r="M5" s="7" t="n">
         <v>34900</v>
       </c>
+      <c r="N5" s="7" t="n">
+        <v>33800</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>33100</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -884,6 +924,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N6" s="9" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -939,6 +987,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N7" s="7" t="n">
+        <v>29400</v>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1006,6 +1062,16 @@
           <t>2026-02-13</t>
         </is>
       </c>
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1049,6 +1115,12 @@
       <c r="M9" s="13" t="n">
         <v>44250</v>
       </c>
+      <c r="N9" s="13" t="n">
+        <v>39950</v>
+      </c>
+      <c r="O9" s="13" t="n">
+        <v>42850</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1092,6 +1164,12 @@
       <c r="M10" s="15" t="n">
         <v>-246.38</v>
       </c>
+      <c r="N10" s="15" t="n">
+        <v>-726.71</v>
+      </c>
+      <c r="O10" s="16" t="n">
+        <v>23.22</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1135,6 +1213,12 @@
       <c r="M11" s="13" t="n">
         <v>48800</v>
       </c>
+      <c r="N11" s="13" t="n">
+        <v>43800</v>
+      </c>
+      <c r="O11" s="13" t="n">
+        <v>48000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1177,6 +1261,12 @@
       </c>
       <c r="M12" s="16" t="n">
         <v>1567.65</v>
+      </c>
+      <c r="N12" s="16" t="n">
+        <v>417.87</v>
+      </c>
+      <c r="O12" s="16" t="n">
+        <v>2450.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-03-17
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -571,6 +571,8 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -621,6 +623,12 @@
         </is>
       </c>
       <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -694,6 +702,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -757,6 +775,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P3" s="7" t="n">
+        <v>26650</v>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -820,6 +846,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P4" s="9" t="n">
+        <v>37550</v>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -869,6 +903,12 @@
       <c r="O5" s="7" t="n">
         <v>33100</v>
       </c>
+      <c r="P5" s="7" t="n">
+        <v>34800</v>
+      </c>
+      <c r="Q5" s="7" t="n">
+        <v>34700</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -932,6 +972,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P6" s="9" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -995,6 +1043,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="P7" s="7" t="n">
+        <v>30500</v>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1072,6 +1128,16 @@
           <t>2026-02-27</t>
         </is>
       </c>
+      <c r="P8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="Q8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1121,6 +1187,12 @@
       <c r="O9" s="13" t="n">
         <v>42850</v>
       </c>
+      <c r="P9" s="13" t="n">
+        <v>41900</v>
+      </c>
+      <c r="Q9" s="13" t="n">
+        <v>43900</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1170,6 +1242,12 @@
       <c r="O10" s="16" t="n">
         <v>23.22</v>
       </c>
+      <c r="P10" s="16" t="n">
+        <v>556.33</v>
+      </c>
+      <c r="Q10" s="16" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1219,6 +1297,12 @@
       <c r="O11" s="13" t="n">
         <v>48000</v>
       </c>
+      <c r="P11" s="13" t="n">
+        <v>46200</v>
+      </c>
+      <c r="Q11" s="13" t="n">
+        <v>50750</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1267,6 +1351,12 @@
       </c>
       <c r="O12" s="16" t="n">
         <v>2450.61</v>
+      </c>
+      <c r="P12" s="16" t="n">
+        <v>2145.58</v>
+      </c>
+      <c r="Q12" s="16" t="n">
+        <v>4129.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-01-20
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -544,12 +544,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +566,12 @@
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -577,6 +585,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -592,6 +610,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D3" s="7" t="n">
+        <v>24100</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -607,6 +633,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D4" s="9" t="n">
+        <v>32400</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -620,6 +654,12 @@
       <c r="C5" s="7" t="n">
         <v>33100</v>
       </c>
+      <c r="D5" s="7" t="n">
+        <v>32000</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>32800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -635,6 +675,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D6" s="9" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -650,6 +698,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D7" s="7" t="n">
+        <v>29000</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -667,6 +723,16 @@
           <t>2024-12-12</t>
         </is>
       </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -680,6 +746,12 @@
       <c r="C9" s="13" t="n">
         <v>41200</v>
       </c>
+      <c r="D9" s="13" t="n">
+        <v>38600</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>41300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -693,6 +765,12 @@
       <c r="C10" s="15" t="n">
         <v>85.70999999999999</v>
       </c>
+      <c r="D10" s="15" t="n">
+        <v>615.92</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>349.01</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -706,6 +784,12 @@
       <c r="C11" s="13" t="n">
         <v>45000</v>
       </c>
+      <c r="D11" s="13" t="n">
+        <v>41300</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>44700</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -718,6 +802,12 @@
       </c>
       <c r="C12" s="15" t="n">
         <v>1176.79</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>632.04</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>1041.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-02-04
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,6 +552,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,6 +574,12 @@
         </is>
       </c>
       <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>2025-02-04</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -595,6 +603,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -618,6 +636,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F3" s="7" t="n">
+        <v>24900</v>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -641,6 +667,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F4" s="9" t="n">
+        <v>33200</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -660,6 +694,12 @@
       <c r="E5" s="7" t="n">
         <v>32800</v>
       </c>
+      <c r="F5" s="7" t="n">
+        <v>32800</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>33700</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -683,6 +723,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F6" s="9" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -706,6 +754,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F7" s="7" t="n">
+        <v>29600</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -733,6 +789,16 @@
           <t>2025-01-20</t>
         </is>
       </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>2025-02-04</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>2025-02-04</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -752,6 +818,12 @@
       <c r="E9" s="13" t="n">
         <v>41300</v>
       </c>
+      <c r="F9" s="13" t="n">
+        <v>39150</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>42100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -771,6 +843,12 @@
       <c r="E10" s="15" t="n">
         <v>349.01</v>
       </c>
+      <c r="F10" s="15" t="n">
+        <v>206.63</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>170.92</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -790,6 +868,12 @@
       <c r="E11" s="13" t="n">
         <v>44700</v>
       </c>
+      <c r="F11" s="13" t="n">
+        <v>42000</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>45800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -808,6 +892,12 @@
       </c>
       <c r="E12" s="15" t="n">
         <v>1041.4</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>1155.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-03-13
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -46,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,6 +183,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -544,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -554,6 +563,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -580,6 +591,12 @@
         </is>
       </c>
       <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-13</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -613,6 +630,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -644,6 +671,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H3" s="7" t="n">
+        <v>25050</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -675,6 +710,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H4" s="9" t="n">
+        <v>36250</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -700,6 +743,12 @@
       <c r="G5" s="7" t="n">
         <v>33700</v>
       </c>
+      <c r="H5" s="7" t="n">
+        <v>33400</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>33200</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -731,6 +780,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H6" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -762,6 +819,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H7" s="7" t="n">
+        <v>29000</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -799,6 +864,16 @@
           <t>2025-02-04</t>
         </is>
       </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>2025-03-13</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>2025-03-13</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -824,6 +899,12 @@
       <c r="G9" s="13" t="n">
         <v>42100</v>
       </c>
+      <c r="H9" s="13" t="n">
+        <v>39900</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>41800</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -849,6 +930,12 @@
       <c r="G10" s="15" t="n">
         <v>170.92</v>
       </c>
+      <c r="H10" s="15" t="n">
+        <v>426.29</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>-352.58</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -874,6 +961,12 @@
       <c r="G11" s="13" t="n">
         <v>45800</v>
       </c>
+      <c r="H11" s="13" t="n">
+        <v>43500</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>47000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -898,6 +991,12 @@
       </c>
       <c r="G12" s="15" t="n">
         <v>1155.49</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>1330.5</v>
+      </c>
+      <c r="I12" s="15" t="n">
+        <v>2130.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-05-05
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -565,6 +565,8 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,6 +599,12 @@
         </is>
       </c>
       <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>2025-05-05</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -640,6 +648,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -679,6 +697,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J3" s="7" t="n">
+        <v>24200</v>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -718,6 +744,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J4" s="9" t="n">
+        <v>34200</v>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -749,6 +783,12 @@
       <c r="I5" s="7" t="n">
         <v>33200</v>
       </c>
+      <c r="J5" s="7" t="n">
+        <v>32700</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>33600</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -788,6 +828,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J6" s="9" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -827,6 +875,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J7" s="7" t="n">
+        <v>28550</v>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -874,6 +930,16 @@
           <t>2025-03-13</t>
         </is>
       </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>2025-05-05</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>2025-05-05</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -905,6 +971,12 @@
       <c r="I9" s="13" t="n">
         <v>41800</v>
       </c>
+      <c r="J9" s="13" t="n">
+        <v>40300</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>42100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -936,6 +1008,12 @@
       <c r="I10" s="16" t="n">
         <v>-352.58</v>
       </c>
+      <c r="J10" s="15" t="n">
+        <v>1969.18</v>
+      </c>
+      <c r="K10" s="15" t="n">
+        <v>441.85</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -967,6 +1045,12 @@
       <c r="I11" s="13" t="n">
         <v>47000</v>
       </c>
+      <c r="J11" s="13" t="n">
+        <v>44300</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>47300</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -997,6 +1081,12 @@
       </c>
       <c r="I12" s="15" t="n">
         <v>2130.2</v>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>3282.54</v>
+      </c>
+      <c r="K12" s="15" t="n">
+        <v>2928.59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-07-03
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,6 +567,8 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +607,12 @@
         </is>
       </c>
       <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -658,6 +666,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -705,6 +723,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L3" s="7" t="n">
+        <v>22550</v>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -752,6 +778,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L4" s="9" t="n">
+        <v>32450</v>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -789,6 +823,12 @@
       <c r="K5" s="7" t="n">
         <v>33600</v>
       </c>
+      <c r="L5" s="7" t="n">
+        <v>30900</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>32300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -836,6 +876,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L6" s="9" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -883,6 +931,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L7" s="7" t="n">
+        <v>26500</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -940,6 +996,16 @@
           <t>2025-05-05</t>
         </is>
       </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -977,6 +1043,12 @@
       <c r="K9" s="13" t="n">
         <v>42100</v>
       </c>
+      <c r="L9" s="13" t="n">
+        <v>36800</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>40400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1014,6 +1086,12 @@
       <c r="K10" s="15" t="n">
         <v>441.85</v>
       </c>
+      <c r="L10" s="15" t="n">
+        <v>498.63</v>
+      </c>
+      <c r="M10" s="15" t="n">
+        <v>408.01</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1051,6 +1129,12 @@
       <c r="K11" s="13" t="n">
         <v>47300</v>
       </c>
+      <c r="L11" s="13" t="n">
+        <v>39900</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>44400</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1087,6 +1171,12 @@
       </c>
       <c r="K12" s="15" t="n">
         <v>2928.59</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>928.22</v>
+      </c>
+      <c r="M12" s="15" t="n">
+        <v>1708.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-07-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -569,6 +569,8 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -613,6 +615,12 @@
         </is>
       </c>
       <c r="M1" s="3" t="n"/>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>2025-07-30</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -676,6 +684,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -731,6 +749,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N3" s="7" t="n">
+        <v>24900</v>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -786,6 +812,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N4" s="9" t="n">
+        <v>33700</v>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -829,6 +863,12 @@
       <c r="M5" s="7" t="n">
         <v>32300</v>
       </c>
+      <c r="N5" s="7" t="n">
+        <v>31500</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>31900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -884,6 +924,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N6" s="9" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -939,6 +987,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="N7" s="7" t="n">
+        <v>28900</v>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1006,6 +1062,16 @@
           <t>2025-07-03</t>
         </is>
       </c>
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>2025-07-30</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
+          <t>2025-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1049,6 +1115,12 @@
       <c r="M9" s="13" t="n">
         <v>40400</v>
       </c>
+      <c r="N9" s="13" t="n">
+        <v>37500</v>
+      </c>
+      <c r="O9" s="13" t="n">
+        <v>40000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1092,6 +1164,12 @@
       <c r="M10" s="15" t="n">
         <v>408.01</v>
       </c>
+      <c r="N10" s="16" t="n">
+        <v>-1301.05</v>
+      </c>
+      <c r="O10" s="16" t="n">
+        <v>-1068.01</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1135,6 +1213,12 @@
       <c r="M11" s="13" t="n">
         <v>44400</v>
       </c>
+      <c r="N11" s="13" t="n">
+        <v>40400</v>
+      </c>
+      <c r="O11" s="13" t="n">
+        <v>44900</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1177,6 +1261,12 @@
       </c>
       <c r="M12" s="15" t="n">
         <v>1708.07</v>
+      </c>
+      <c r="N12" s="16" t="n">
+        <v>-1091.46</v>
+      </c>
+      <c r="O12" s="15" t="n">
+        <v>1123.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-04-02
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AI12"/>
+  <dimension ref="A1:AK12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -591,6 +591,8 @@
     <col width="14" customWidth="1" min="33" max="33"/>
     <col width="14" customWidth="1" min="34" max="34"/>
     <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="14" customWidth="1" min="36" max="36"/>
+    <col width="14" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -701,6 +703,12 @@
         </is>
       </c>
       <c r="AI1" s="3" t="n"/>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="AK1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -874,6 +882,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="AJ2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="AK2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1017,6 +1035,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AJ3" s="7" t="n">
+        <v>27400</v>
+      </c>
+      <c r="AK3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1160,6 +1186,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AJ4" s="9" t="n">
+        <v>38550</v>
+      </c>
+      <c r="AK4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1269,6 +1303,12 @@
       <c r="AI5" s="7" t="n">
         <v>34500</v>
       </c>
+      <c r="AJ5" s="7" t="n">
+        <v>36000</v>
+      </c>
+      <c r="AK5" s="7" t="n">
+        <v>36500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1412,6 +1452,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AJ6" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="AK6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -1555,6 +1603,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AJ7" s="7" t="n">
+        <v>31400</v>
+      </c>
+      <c r="AK7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1732,6 +1788,16 @@
           <t>2026-03-26</t>
         </is>
       </c>
+      <c r="AJ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="AK8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1841,6 +1907,12 @@
       <c r="AI9" s="13" t="n">
         <v>43250</v>
       </c>
+      <c r="AJ9" s="13" t="n">
+        <v>42850</v>
+      </c>
+      <c r="AK9" s="13" t="n">
+        <v>45500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1950,6 +2022,12 @@
       <c r="AI10" s="15" t="n">
         <v>65.27</v>
       </c>
+      <c r="AJ10" s="15" t="n">
+        <v>416.63</v>
+      </c>
+      <c r="AK10" s="15" t="n">
+        <v>92.68000000000001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -2059,6 +2137,12 @@
       <c r="AI11" s="13" t="n">
         <v>49500</v>
       </c>
+      <c r="AJ11" s="13" t="n">
+        <v>48200</v>
+      </c>
+      <c r="AK11" s="13" t="n">
+        <v>52950</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -2167,6 +2251,12 @@
       </c>
       <c r="AI12" s="15" t="n">
         <v>3589.8</v>
+      </c>
+      <c r="AJ12" s="15" t="n">
+        <v>3047.16</v>
+      </c>
+      <c r="AK12" s="15" t="n">
+        <v>4799.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-07-31
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -46,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,6 +183,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -544,12 +553,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +575,12 @@
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -577,6 +594,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -592,6 +619,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D3" s="7" t="n">
+        <v>24800</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -607,6 +642,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D4" s="9" t="n">
+        <v>33700</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -620,6 +663,12 @@
       <c r="C5" s="7" t="n">
         <v>32800</v>
       </c>
+      <c r="D5" s="7" t="n">
+        <v>31200</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>31900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -635,6 +684,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D6" s="9" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -650,6 +707,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D7" s="7" t="n">
+        <v>28800</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -667,6 +732,16 @@
           <t>2025-05-30</t>
         </is>
       </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -680,6 +755,12 @@
       <c r="C9" s="13" t="n">
         <v>41200</v>
       </c>
+      <c r="D9" s="13" t="n">
+        <v>37500</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>40100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -693,6 +774,12 @@
       <c r="C10" s="15" t="n">
         <v>318.45</v>
       </c>
+      <c r="D10" s="16" t="n">
+        <v>-1172.9</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>-919.91</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -706,6 +793,12 @@
       <c r="C11" s="13" t="n">
         <v>45800</v>
       </c>
+      <c r="D11" s="13" t="n">
+        <v>40200</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>44700</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -718,6 +811,12 @@
       </c>
       <c r="C12" s="15" t="n">
         <v>2211.4</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>-1162.28</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>971.9299999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-09-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -561,6 +561,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -581,6 +583,12 @@
         </is>
       </c>
       <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -604,6 +612,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -627,6 +645,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F3" s="7" t="n">
+        <v>24300</v>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -650,6 +676,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F4" s="9" t="n">
+        <v>32850</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -669,6 +703,12 @@
       <c r="E5" s="7" t="n">
         <v>31900</v>
       </c>
+      <c r="F5" s="7" t="n">
+        <v>31800</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>31400</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -692,6 +732,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F6" s="9" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -715,6 +763,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F7" s="7" t="n">
+        <v>28450</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -742,6 +798,16 @@
           <t>2025-07-31</t>
         </is>
       </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -761,6 +827,12 @@
       <c r="E9" s="13" t="n">
         <v>40100</v>
       </c>
+      <c r="F9" s="13" t="n">
+        <v>36350</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>39300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -780,6 +852,12 @@
       <c r="E10" s="16" t="n">
         <v>-919.91</v>
       </c>
+      <c r="F10" s="16" t="n">
+        <v>-1776.62</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>-1076.88</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -799,6 +877,12 @@
       <c r="E11" s="13" t="n">
         <v>44700</v>
       </c>
+      <c r="F11" s="13" t="n">
+        <v>39400</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>42800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -817,6 +901,12 @@
       </c>
       <c r="E12" s="15" t="n">
         <v>971.9299999999999</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>-1411.63</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>-279.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-01-31
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,6 +591,12 @@
         </is>
       </c>
       <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -622,6 +630,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -653,6 +671,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H3" s="7" t="n">
+        <v>25750</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -684,6 +710,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H4" s="9" t="n">
+        <v>38150</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -709,6 +743,12 @@
       <c r="G5" s="7" t="n">
         <v>31400</v>
       </c>
+      <c r="H5" s="7" t="n">
+        <v>33750</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>34400</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -740,6 +780,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H6" s="9" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -771,6 +819,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H7" s="7" t="n">
+        <v>29150</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -808,6 +864,16 @@
           <t>2025-09-30</t>
         </is>
       </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -833,6 +899,12 @@
       <c r="G9" s="13" t="n">
         <v>39300</v>
       </c>
+      <c r="H9" s="13" t="n">
+        <v>40800</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>44100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -858,6 +930,12 @@
       <c r="G10" s="16" t="n">
         <v>-1076.88</v>
       </c>
+      <c r="H10" s="15" t="n">
+        <v>433.02</v>
+      </c>
+      <c r="I10" s="15" t="n">
+        <v>741.76</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -883,6 +961,12 @@
       <c r="G11" s="13" t="n">
         <v>42800</v>
       </c>
+      <c r="H11" s="13" t="n">
+        <v>44200</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>48300</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -907,6 +991,12 @@
       </c>
       <c r="G12" s="16" t="n">
         <v>-279.89</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>1130.09</v>
+      </c>
+      <c r="I12" s="15" t="n">
+        <v>2214.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2024-12-12
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -565,6 +565,8 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,6 +599,12 @@
         </is>
       </c>
       <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>2024-12-12</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -640,6 +648,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -679,6 +697,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J3" s="7" t="n">
+        <v>24200</v>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -718,6 +744,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J4" s="9" t="n">
+        <v>32550</v>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -749,6 +783,12 @@
       <c r="I5" s="7" t="n">
         <v>34400</v>
       </c>
+      <c r="J5" s="7" t="n">
+        <v>31300</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>33100</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -788,6 +828,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J6" s="9" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -827,6 +875,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J7" s="7" t="n">
+        <v>28800</v>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -874,6 +930,16 @@
           <t>2026-01-31</t>
         </is>
       </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>2024-12-12</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>2024-12-12</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -905,6 +971,12 @@
       <c r="I9" s="13" t="n">
         <v>44100</v>
       </c>
+      <c r="J9" s="13" t="n">
+        <v>38450</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>41200</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -936,6 +1008,12 @@
       <c r="I10" s="15" t="n">
         <v>741.76</v>
       </c>
+      <c r="J10" s="15" t="n">
+        <v>518.6900000000001</v>
+      </c>
+      <c r="K10" s="15" t="n">
+        <v>85.70999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -967,6 +1045,12 @@
       <c r="I11" s="13" t="n">
         <v>48300</v>
       </c>
+      <c r="J11" s="13" t="n">
+        <v>41400</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>45000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -997,6 +1081,12 @@
       </c>
       <c r="I12" s="15" t="n">
         <v>2214.89</v>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>785.24</v>
+      </c>
+      <c r="K12" s="15" t="n">
+        <v>1176.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-05-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,6 +567,8 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +607,12 @@
         </is>
       </c>
       <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -658,6 +666,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -705,6 +723,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L3" s="7" t="n">
+        <v>23700</v>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -752,6 +778,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L4" s="9" t="n">
+        <v>33100</v>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -789,6 +823,12 @@
       <c r="K5" s="7" t="n">
         <v>33600</v>
       </c>
+      <c r="L5" s="7" t="n">
+        <v>31800</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>32800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -836,6 +876,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L6" s="9" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -883,6 +931,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L7" s="7" t="n">
+        <v>27700</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -940,6 +996,16 @@
           <t>2025-05-05</t>
         </is>
       </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -977,6 +1043,12 @@
       <c r="K9" s="13" t="n">
         <v>42100</v>
       </c>
+      <c r="L9" s="13" t="n">
+        <v>39050</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>41200</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1014,6 +1086,12 @@
       <c r="K10" s="15" t="n">
         <v>441.85</v>
       </c>
+      <c r="L10" s="15" t="n">
+        <v>1458.55</v>
+      </c>
+      <c r="M10" s="15" t="n">
+        <v>318.45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1051,6 +1129,12 @@
       <c r="K11" s="13" t="n">
         <v>47300</v>
       </c>
+      <c r="L11" s="13" t="n">
+        <v>42500</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>45800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -1087,6 +1171,12 @@
       </c>
       <c r="K12" s="15" t="n">
         <v>2928.59</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>2227.82</v>
+      </c>
+      <c r="M12" s="15" t="n">
+        <v>2211.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-08-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -46,7 +46,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,6 +183,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -544,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,6 +561,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,6 +583,12 @@
         </is>
       </c>
       <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -595,6 +612,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -618,6 +645,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F3" s="7" t="n">
+        <v>23150</v>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -641,6 +676,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F4" s="9" t="n">
+        <v>33250</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -660,6 +703,12 @@
       <c r="E5" s="7" t="n">
         <v>32400</v>
       </c>
+      <c r="F5" s="7" t="n">
+        <v>31500</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>30700</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -683,6 +732,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F6" s="9" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -706,6 +763,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="F7" s="7" t="n">
+        <v>27750</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -733,6 +798,16 @@
           <t>2025-06-28</t>
         </is>
       </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -752,6 +827,12 @@
       <c r="E9" s="13" t="n">
         <v>40500</v>
       </c>
+      <c r="F9" s="13" t="n">
+        <v>36600</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>38900</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -771,6 +852,12 @@
       <c r="E10" s="15" t="n">
         <v>544.96</v>
       </c>
+      <c r="F10" s="16" t="n">
+        <v>-485.6</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>-610.1900000000001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -790,6 +877,12 @@
       <c r="E11" s="13" t="n">
         <v>44700</v>
       </c>
+      <c r="F11" s="13" t="n">
+        <v>39500</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>42400</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -808,6 +901,12 @@
       </c>
       <c r="E12" s="15" t="n">
         <v>2045.32</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>-262.29</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>193.73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-06-28
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -544,12 +544,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +566,12 @@
         </is>
       </c>
       <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>2025-06-28</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -577,6 +585,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -592,6 +610,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D3" s="7" t="n">
+        <v>22350</v>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -607,6 +633,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D4" s="9" t="n">
+        <v>32550</v>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -620,6 +654,12 @@
       <c r="C5" s="7" t="n">
         <v>33800</v>
       </c>
+      <c r="D5" s="7" t="n">
+        <v>31100</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>32400</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -635,6 +675,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D6" s="9" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -650,6 +698,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="D7" s="7" t="n">
+        <v>26400</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -667,6 +723,16 @@
           <t>2025-04-30</t>
         </is>
       </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>2025-06-28</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>2025-06-28</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -680,6 +746,12 @@
       <c r="C9" s="13" t="n">
         <v>42250</v>
       </c>
+      <c r="D9" s="13" t="n">
+        <v>37050</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>40500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -693,6 +765,12 @@
       <c r="C10" s="15" t="n">
         <v>169.18</v>
       </c>
+      <c r="D10" s="15" t="n">
+        <v>902.54</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>544.96</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -706,6 +784,12 @@
       <c r="C11" s="13" t="n">
         <v>47800</v>
       </c>
+      <c r="D11" s="13" t="n">
+        <v>40400</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>44700</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -718,6 +802,12 @@
       </c>
       <c r="C12" s="15" t="n">
         <v>3002.54</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>1583.36</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>2045.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-03-28
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,8 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,6 +591,12 @@
         </is>
       </c>
       <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -622,6 +630,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -653,6 +671,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H3" s="7" t="n">
+        <v>25800</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -684,6 +710,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H4" s="9" t="n">
+        <v>37050</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -709,6 +743,12 @@
       <c r="G5" s="7" t="n">
         <v>30700</v>
       </c>
+      <c r="H5" s="7" t="n">
+        <v>34500</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>34500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -740,6 +780,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H6" s="9" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -771,6 +819,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H7" s="7" t="n">
+        <v>29650</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -808,6 +864,16 @@
           <t>2025-08-30</t>
         </is>
       </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -833,6 +899,12 @@
       <c r="G9" s="13" t="n">
         <v>38900</v>
       </c>
+      <c r="H9" s="13" t="n">
+        <v>40950</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>43500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -858,6 +930,12 @@
       <c r="G10" s="16" t="n">
         <v>-610.1900000000001</v>
       </c>
+      <c r="H10" s="15" t="n">
+        <v>509.7</v>
+      </c>
+      <c r="I10" s="15" t="n">
+        <v>172.45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -883,6 +961,12 @@
       <c r="G11" s="13" t="n">
         <v>42400</v>
       </c>
+      <c r="H11" s="13" t="n">
+        <v>45600</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>50300</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -907,6 +991,12 @@
       </c>
       <c r="G12" s="15" t="n">
         <v>193.73</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>2456.18</v>
+      </c>
+      <c r="I12" s="15" t="n">
+        <v>4245.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-04-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -565,6 +565,8 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,6 +599,12 @@
         </is>
       </c>
       <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -640,6 +648,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -679,6 +697,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J3" s="7" t="n">
+        <v>24700</v>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -718,6 +744,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J4" s="9" t="n">
+        <v>34800</v>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -749,6 +783,12 @@
       <c r="I5" s="7" t="n">
         <v>33200</v>
       </c>
+      <c r="J5" s="7" t="n">
+        <v>32700</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>33800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -788,6 +828,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J6" s="9" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -827,6 +875,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="J7" s="7" t="n">
+        <v>29000</v>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -874,6 +930,16 @@
           <t>2025-03-13</t>
         </is>
       </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -905,6 +971,12 @@
       <c r="I9" s="13" t="n">
         <v>41800</v>
       </c>
+      <c r="J9" s="13" t="n">
+        <v>40500</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>42250</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -936,6 +1008,12 @@
       <c r="I10" s="16" t="n">
         <v>-352.58</v>
       </c>
+      <c r="J10" s="15" t="n">
+        <v>1612.62</v>
+      </c>
+      <c r="K10" s="15" t="n">
+        <v>169.18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -967,6 +1045,12 @@
       <c r="I11" s="13" t="n">
         <v>47000</v>
       </c>
+      <c r="J11" s="13" t="n">
+        <v>44800</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>47800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -997,6 +1081,12 @@
       </c>
       <c r="I12" s="15" t="n">
         <v>2130.2</v>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>3221.52</v>
+      </c>
+      <c r="K12" s="15" t="n">
+        <v>3002.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2025-12-19
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BA12"/>
+  <dimension ref="A1:BC12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -609,6 +609,8 @@
     <col width="14" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="55" max="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -773,6 +775,12 @@
         </is>
       </c>
       <c r="BA1" s="3" t="n"/>
+      <c r="BB1" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="BC1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1036,6 +1044,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BB2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BC2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1251,6 +1269,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BB3" s="7" t="n">
+        <v>22550</v>
+      </c>
+      <c r="BC3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1466,6 +1492,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BB4" s="9" t="n">
+        <v>33000</v>
+      </c>
+      <c r="BC4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1629,6 +1663,12 @@
       <c r="BA5" s="7" t="n">
         <v>36500</v>
       </c>
+      <c r="BB5" s="7" t="n">
+        <v>31300</v>
+      </c>
+      <c r="BC5" s="7" t="n">
+        <v>31300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1844,6 +1884,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BB6" s="9" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="BC6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2059,6 +2107,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BB7" s="7" t="n">
+        <v>26550</v>
+      </c>
+      <c r="BC7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2326,6 +2382,16 @@
           <t>2026-04-02</t>
         </is>
       </c>
+      <c r="BB8" s="11" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="BC8" s="11" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2489,6 +2555,12 @@
       <c r="BA9" s="13" t="n">
         <v>45500</v>
       </c>
+      <c r="BB9" s="13" t="n">
+        <v>36800</v>
+      </c>
+      <c r="BC9" s="13" t="n">
+        <v>39400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -2652,6 +2724,12 @@
       <c r="BA10" s="15" t="n">
         <v>92.68000000000001</v>
       </c>
+      <c r="BB10" s="15" t="n">
+        <v>427</v>
+      </c>
+      <c r="BC10" s="16" t="n">
+        <v>-95.17</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -2815,6 +2893,12 @@
       <c r="BA11" s="13" t="n">
         <v>52950</v>
       </c>
+      <c r="BB11" s="13" t="n">
+        <v>39600</v>
+      </c>
+      <c r="BC11" s="13" t="n">
+        <v>42500</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -2977,6 +3061,12 @@
       </c>
       <c r="BA12" s="15" t="n">
         <v>4799.42</v>
+      </c>
+      <c r="BB12" s="15" t="n">
+        <v>556.02</v>
+      </c>
+      <c r="BC12" s="15" t="n">
+        <v>308.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-02-28
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BC12"/>
+  <dimension ref="A1:BE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -611,6 +611,8 @@
     <col width="14" customWidth="1" min="53" max="53"/>
     <col width="14" customWidth="1" min="54" max="54"/>
     <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -781,6 +783,12 @@
         </is>
       </c>
       <c r="BC1" s="3" t="n"/>
+      <c r="BD1" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="BE1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1054,6 +1062,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BD2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BE2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1277,6 +1295,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BD3" s="7" t="n">
+        <v>25800</v>
+      </c>
+      <c r="BE3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1500,6 +1526,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BD4" s="9" t="n">
+        <v>37800</v>
+      </c>
+      <c r="BE4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1669,6 +1703,12 @@
       <c r="BC5" s="7" t="n">
         <v>31300</v>
       </c>
+      <c r="BD5" s="7" t="n">
+        <v>33700</v>
+      </c>
+      <c r="BE5" s="7" t="n">
+        <v>32800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1892,6 +1932,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BD6" s="9" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="BE6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2115,6 +2163,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BD7" s="7" t="n">
+        <v>29150</v>
+      </c>
+      <c r="BE7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2392,6 +2448,16 @@
           <t>2025-12-19</t>
         </is>
       </c>
+      <c r="BD8" s="11" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="BE8" s="11" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2561,6 +2627,12 @@
       <c r="BC9" s="13" t="n">
         <v>39400</v>
       </c>
+      <c r="BD9" s="13" t="n">
+        <v>39750</v>
+      </c>
+      <c r="BE9" s="13" t="n">
+        <v>42400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -2730,6 +2802,12 @@
       <c r="BC10" s="16" t="n">
         <v>-95.17</v>
       </c>
+      <c r="BD10" s="16" t="n">
+        <v>-610.99</v>
+      </c>
+      <c r="BE10" s="16" t="n">
+        <v>-105.68</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -2899,6 +2977,12 @@
       <c r="BC11" s="13" t="n">
         <v>42500</v>
       </c>
+      <c r="BD11" s="13" t="n">
+        <v>43600</v>
+      </c>
+      <c r="BE11" s="13" t="n">
+        <v>48000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3067,6 +3151,12 @@
       </c>
       <c r="BC12" s="15" t="n">
         <v>308.87</v>
+      </c>
+      <c r="BD12" s="15" t="n">
+        <v>536.13</v>
+      </c>
+      <c r="BE12" s="15" t="n">
+        <v>2774.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-04-10
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BE12"/>
+  <dimension ref="A1:BG12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -613,6 +613,8 @@
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="14" customWidth="1" min="56" max="56"/>
     <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
+    <col width="14" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -789,6 +791,12 @@
         </is>
       </c>
       <c r="BE1" s="3" t="n"/>
+      <c r="BF1" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="BG1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1072,6 +1080,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BF2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BG2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1303,6 +1321,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BF3" s="7" t="n">
+        <v>27050</v>
+      </c>
+      <c r="BG3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1534,6 +1560,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BF4" s="9" t="n">
+        <v>39700</v>
+      </c>
+      <c r="BG4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1709,6 +1743,12 @@
       <c r="BE5" s="7" t="n">
         <v>36500</v>
       </c>
+      <c r="BF5" s="7" t="n">
+        <v>36300</v>
+      </c>
+      <c r="BG5" s="7" t="n">
+        <v>37300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1940,6 +1980,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BF6" s="9" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="BG6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2171,6 +2219,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BF7" s="7" t="n">
+        <v>31000</v>
+      </c>
+      <c r="BG7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2458,6 +2514,16 @@
           <t>2026-04-02</t>
         </is>
       </c>
+      <c r="BF8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="BG8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2633,6 +2699,12 @@
       <c r="BE9" s="13" t="n">
         <v>45500</v>
       </c>
+      <c r="BF9" s="13" t="n">
+        <v>43100</v>
+      </c>
+      <c r="BG9" s="13" t="n">
+        <v>46400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -2808,6 +2880,12 @@
       <c r="BE10" s="15" t="n">
         <v>92.68000000000001</v>
       </c>
+      <c r="BF10" s="15" t="n">
+        <v>748.29</v>
+      </c>
+      <c r="BG10" s="15" t="n">
+        <v>512.16</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -2983,6 +3061,12 @@
       <c r="BE11" s="13" t="n">
         <v>52950</v>
       </c>
+      <c r="BF11" s="13" t="n">
+        <v>47800</v>
+      </c>
+      <c r="BG11" s="13" t="n">
+        <v>53550</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3157,6 +3241,12 @@
       </c>
       <c r="BE12" s="15" t="n">
         <v>4799.42</v>
+      </c>
+      <c r="BF12" s="15" t="n">
+        <v>2729.48</v>
+      </c>
+      <c r="BG12" s="15" t="n">
+        <v>4915.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-04-16
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BG12"/>
+  <dimension ref="A1:BI12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -615,6 +615,8 @@
     <col width="14" customWidth="1" min="57" max="57"/>
     <col width="14" customWidth="1" min="58" max="58"/>
     <col width="14" customWidth="1" min="59" max="59"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
+    <col width="14" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -797,6 +799,12 @@
         </is>
       </c>
       <c r="BG1" s="3" t="n"/>
+      <c r="BH1" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="BI1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1090,6 +1098,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BH2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BI2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1329,6 +1347,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BH3" s="7" t="n">
+        <v>26200</v>
+      </c>
+      <c r="BI3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1568,6 +1594,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BH4" s="9" t="n">
+        <v>39600</v>
+      </c>
+      <c r="BI4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1749,6 +1783,12 @@
       <c r="BG5" s="7" t="n">
         <v>37300</v>
       </c>
+      <c r="BH5" s="7" t="n">
+        <v>35800</v>
+      </c>
+      <c r="BI5" s="7" t="n">
+        <v>36100</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1988,6 +2028,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BH6" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="BI6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2227,6 +2275,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BH7" s="7" t="n">
+        <v>29900</v>
+      </c>
+      <c r="BI7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2524,6 +2580,16 @@
           <t>2026-04-10</t>
         </is>
       </c>
+      <c r="BH8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="BI8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2705,6 +2771,12 @@
       <c r="BG9" s="13" t="n">
         <v>46400</v>
       </c>
+      <c r="BH9" s="13" t="n">
+        <v>42200</v>
+      </c>
+      <c r="BI9" s="13" t="n">
+        <v>45300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -2886,6 +2958,12 @@
       <c r="BG10" s="15" t="n">
         <v>512.16</v>
       </c>
+      <c r="BH10" s="15" t="n">
+        <v>809.99</v>
+      </c>
+      <c r="BI10" s="15" t="n">
+        <v>502.18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3067,6 +3145,12 @@
       <c r="BG11" s="13" t="n">
         <v>53550</v>
       </c>
+      <c r="BH11" s="13" t="n">
+        <v>46900</v>
+      </c>
+      <c r="BI11" s="13" t="n">
+        <v>51150</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3247,6 +3331,12 @@
       </c>
       <c r="BG12" s="15" t="n">
         <v>4915.05</v>
+      </c>
+      <c r="BH12" s="15" t="n">
+        <v>2798.87</v>
+      </c>
+      <c r="BI12" s="15" t="n">
+        <v>3613.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-04-23
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BI12"/>
+  <dimension ref="A1:BK12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -617,6 +617,8 @@
     <col width="14" customWidth="1" min="59" max="59"/>
     <col width="14" customWidth="1" min="60" max="60"/>
     <col width="14" customWidth="1" min="61" max="61"/>
+    <col width="14" customWidth="1" min="62" max="62"/>
+    <col width="14" customWidth="1" min="63" max="63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -805,6 +807,12 @@
         </is>
       </c>
       <c r="BI1" s="3" t="n"/>
+      <c r="BJ1" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="BK1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1108,6 +1116,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BJ2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BK2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1355,6 +1373,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BJ3" s="7" t="n">
+        <v>26300</v>
+      </c>
+      <c r="BK3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1602,6 +1628,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BJ4" s="9" t="n">
+        <v>39600</v>
+      </c>
+      <c r="BK4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1789,6 +1823,12 @@
       <c r="BI5" s="7" t="n">
         <v>36100</v>
       </c>
+      <c r="BJ5" s="7" t="n">
+        <v>35700</v>
+      </c>
+      <c r="BK5" s="7" t="n">
+        <v>35600</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2036,6 +2076,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BJ6" s="9" t="n">
+        <v>82.7</v>
+      </c>
+      <c r="BK6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2283,6 +2331,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BJ7" s="7" t="n">
+        <v>30250</v>
+      </c>
+      <c r="BK7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2590,6 +2646,16 @@
           <t>2026-04-16</t>
         </is>
       </c>
+      <c r="BJ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="BK8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2777,6 +2843,12 @@
       <c r="BI9" s="13" t="n">
         <v>45300</v>
       </c>
+      <c r="BJ9" s="13" t="n">
+        <v>42450</v>
+      </c>
+      <c r="BK9" s="13" t="n">
+        <v>44700</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -2964,6 +3036,12 @@
       <c r="BI10" s="15" t="n">
         <v>502.18</v>
       </c>
+      <c r="BJ10" s="15" t="n">
+        <v>961.9400000000001</v>
+      </c>
+      <c r="BK10" s="15" t="n">
+        <v>132.7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3151,6 +3229,12 @@
       <c r="BI11" s="13" t="n">
         <v>51150</v>
       </c>
+      <c r="BJ11" s="13" t="n">
+        <v>46700</v>
+      </c>
+      <c r="BK11" s="13" t="n">
+        <v>50200</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3337,6 +3421,12 @@
       </c>
       <c r="BI12" s="15" t="n">
         <v>3613.8</v>
+      </c>
+      <c r="BJ12" s="15" t="n">
+        <v>2500.04</v>
+      </c>
+      <c r="BK12" s="15" t="n">
+        <v>2896.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-04-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BK12"/>
+  <dimension ref="A1:BM12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -619,6 +619,8 @@
     <col width="14" customWidth="1" min="61" max="61"/>
     <col width="14" customWidth="1" min="62" max="62"/>
     <col width="14" customWidth="1" min="63" max="63"/>
+    <col width="14" customWidth="1" min="64" max="64"/>
+    <col width="14" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,6 +815,12 @@
         </is>
       </c>
       <c r="BK1" s="3" t="n"/>
+      <c r="BL1" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="BM1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1126,6 +1134,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BL2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BM2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1381,6 +1399,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BL3" s="7" t="n">
+        <v>25550</v>
+      </c>
+      <c r="BM3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1636,6 +1662,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BL4" s="9" t="n">
+        <v>39700</v>
+      </c>
+      <c r="BM4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1829,6 +1863,12 @@
       <c r="BK5" s="7" t="n">
         <v>35600</v>
       </c>
+      <c r="BL5" s="7" t="n">
+        <v>35600</v>
+      </c>
+      <c r="BM5" s="7" t="n">
+        <v>35800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2084,6 +2124,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BL6" s="9" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="BM6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2339,6 +2387,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BL7" s="7" t="n">
+        <v>29800</v>
+      </c>
+      <c r="BM7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2656,6 +2712,16 @@
           <t>2026-04-23</t>
         </is>
       </c>
+      <c r="BL8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="BM8" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2849,6 +2915,12 @@
       <c r="BK9" s="13" t="n">
         <v>44700</v>
       </c>
+      <c r="BL9" s="13" t="n">
+        <v>42000</v>
+      </c>
+      <c r="BM9" s="13" t="n">
+        <v>44500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3042,6 +3114,12 @@
       <c r="BK10" s="15" t="n">
         <v>132.7</v>
       </c>
+      <c r="BL10" s="15" t="n">
+        <v>1241.26</v>
+      </c>
+      <c r="BM10" s="15" t="n">
+        <v>217.12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3235,6 +3313,12 @@
       <c r="BK11" s="13" t="n">
         <v>50200</v>
       </c>
+      <c r="BL11" s="13" t="n">
+        <v>46100</v>
+      </c>
+      <c r="BM11" s="13" t="n">
+        <v>49050</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3427,6 +3511,12 @@
       </c>
       <c r="BK12" s="15" t="n">
         <v>2896.16</v>
+      </c>
+      <c r="BL12" s="15" t="n">
+        <v>2635.19</v>
+      </c>
+      <c r="BM12" s="15" t="n">
+        <v>2032.86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-05-07
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BM12"/>
+  <dimension ref="A1:BO12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -621,6 +621,8 @@
     <col width="14" customWidth="1" min="63" max="63"/>
     <col width="14" customWidth="1" min="64" max="64"/>
     <col width="14" customWidth="1" min="65" max="65"/>
+    <col width="14" customWidth="1" min="66" max="66"/>
+    <col width="14" customWidth="1" min="67" max="67"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -821,6 +823,12 @@
         </is>
       </c>
       <c r="BM1" s="3" t="n"/>
+      <c r="BN1" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="BO1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1144,6 +1152,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BN2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BO2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1407,6 +1425,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BN3" s="7" t="n">
+        <v>25850</v>
+      </c>
+      <c r="BO3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1670,6 +1696,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BN4" s="9" t="n">
+        <v>39500</v>
+      </c>
+      <c r="BO4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1869,6 +1903,12 @@
       <c r="BM5" s="7" t="n">
         <v>35800</v>
       </c>
+      <c r="BN5" s="7" t="n">
+        <v>35600</v>
+      </c>
+      <c r="BO5" s="7" t="n">
+        <v>36300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2132,6 +2172,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BN6" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="BO6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2395,6 +2443,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BN7" s="7" t="n">
+        <v>29900</v>
+      </c>
+      <c r="BO7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2722,6 +2778,16 @@
           <t>2026-04-30</t>
         </is>
       </c>
+      <c r="BN8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="BO8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2921,6 +2987,12 @@
       <c r="BM9" s="13" t="n">
         <v>44500</v>
       </c>
+      <c r="BN9" s="13" t="n">
+        <v>41650</v>
+      </c>
+      <c r="BO9" s="13" t="n">
+        <v>44400</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3120,6 +3192,12 @@
       <c r="BM10" s="15" t="n">
         <v>217.12</v>
       </c>
+      <c r="BN10" s="15" t="n">
+        <v>689.09</v>
+      </c>
+      <c r="BO10" s="16" t="n">
+        <v>-222.86</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3319,6 +3397,12 @@
       <c r="BM11" s="13" t="n">
         <v>49050</v>
       </c>
+      <c r="BN11" s="13" t="n">
+        <v>45400</v>
+      </c>
+      <c r="BO11" s="13" t="n">
+        <v>49200</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3517,6 +3601,12 @@
       </c>
       <c r="BM12" s="15" t="n">
         <v>2032.86</v>
+      </c>
+      <c r="BN12" s="15" t="n">
+        <v>1731.4</v>
+      </c>
+      <c r="BO12" s="15" t="n">
+        <v>1840.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-05-14
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BO12"/>
+  <dimension ref="A1:BQ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,8 @@
     <col width="14" customWidth="1" min="65" max="65"/>
     <col width="14" customWidth="1" min="66" max="66"/>
     <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="14" customWidth="1" min="68" max="68"/>
+    <col width="14" customWidth="1" min="69" max="69"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -829,6 +831,12 @@
         </is>
       </c>
       <c r="BO1" s="3" t="n"/>
+      <c r="BP1" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="BQ1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1162,6 +1170,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BP2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BQ2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1433,6 +1451,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BP3" s="7" t="n">
+        <v>25200</v>
+      </c>
+      <c r="BQ3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1704,6 +1730,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BP4" s="9" t="n">
+        <v>39000</v>
+      </c>
+      <c r="BQ4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1909,6 +1943,12 @@
       <c r="BO5" s="7" t="n">
         <v>36300</v>
       </c>
+      <c r="BP5" s="7" t="n">
+        <v>35100</v>
+      </c>
+      <c r="BQ5" s="7" t="n">
+        <v>34800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2180,6 +2220,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BP6" s="9" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="BQ6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2451,6 +2499,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BP7" s="7" t="n">
+        <v>29350</v>
+      </c>
+      <c r="BQ7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2788,6 +2844,16 @@
           <t>2026-05-07</t>
         </is>
       </c>
+      <c r="BP8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="BQ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2993,6 +3059,12 @@
       <c r="BO9" s="13" t="n">
         <v>44400</v>
       </c>
+      <c r="BP9" s="13" t="n">
+        <v>39850</v>
+      </c>
+      <c r="BQ9" s="13" t="n">
+        <v>43000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3198,6 +3270,12 @@
       <c r="BO10" s="16" t="n">
         <v>-222.86</v>
       </c>
+      <c r="BP10" s="16" t="n">
+        <v>-360.22</v>
+      </c>
+      <c r="BQ10" s="16" t="n">
+        <v>-448.33</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3403,6 +3481,12 @@
       <c r="BO11" s="13" t="n">
         <v>49200</v>
       </c>
+      <c r="BP11" s="13" t="n">
+        <v>43400</v>
+      </c>
+      <c r="BQ11" s="13" t="n">
+        <v>47400</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3607,6 +3691,12 @@
       </c>
       <c r="BO12" s="15" t="n">
         <v>1840.15</v>
+      </c>
+      <c r="BP12" s="15" t="n">
+        <v>488.1</v>
+      </c>
+      <c r="BQ12" s="15" t="n">
+        <v>1224.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-05-21
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BQ12"/>
+  <dimension ref="A1:BS12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -625,6 +625,8 @@
     <col width="14" customWidth="1" min="67" max="67"/>
     <col width="14" customWidth="1" min="68" max="68"/>
     <col width="14" customWidth="1" min="69" max="69"/>
+    <col width="14" customWidth="1" min="70" max="70"/>
+    <col width="14" customWidth="1" min="71" max="71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -837,6 +839,12 @@
         </is>
       </c>
       <c r="BQ1" s="3" t="n"/>
+      <c r="BR1" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="BS1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1180,6 +1188,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BR2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BS2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1459,6 +1477,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BR3" s="7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="BS3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1738,6 +1764,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BR4" s="9" t="n">
+        <v>38950</v>
+      </c>
+      <c r="BS4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1949,6 +1983,12 @@
       <c r="BQ5" s="7" t="n">
         <v>34800</v>
       </c>
+      <c r="BR5" s="7" t="n">
+        <v>34500</v>
+      </c>
+      <c r="BS5" s="7" t="n">
+        <v>34200</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2228,6 +2268,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BR6" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="BS6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2507,6 +2555,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BR7" s="7" t="n">
+        <v>29250</v>
+      </c>
+      <c r="BS7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2854,6 +2910,16 @@
           <t>2026-05-14</t>
         </is>
       </c>
+      <c r="BR8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="BS8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3065,6 +3131,12 @@
       <c r="BQ9" s="13" t="n">
         <v>43000</v>
       </c>
+      <c r="BR9" s="13" t="n">
+        <v>39250</v>
+      </c>
+      <c r="BS9" s="13" t="n">
+        <v>42350</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3276,6 +3348,12 @@
       <c r="BQ10" s="16" t="n">
         <v>-448.33</v>
       </c>
+      <c r="BR10" s="16" t="n">
+        <v>-698.23</v>
+      </c>
+      <c r="BS10" s="16" t="n">
+        <v>-672.04</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3487,6 +3565,12 @@
       <c r="BQ11" s="13" t="n">
         <v>47400</v>
       </c>
+      <c r="BR11" s="13" t="n">
+        <v>42300</v>
+      </c>
+      <c r="BS11" s="13" t="n">
+        <v>46350</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3697,6 +3781,12 @@
       </c>
       <c r="BQ12" s="15" t="n">
         <v>1224.09</v>
+      </c>
+      <c r="BR12" s="16" t="n">
+        <v>-347.82</v>
+      </c>
+      <c r="BS12" s="15" t="n">
+        <v>603.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-05-25
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BS12"/>
+  <dimension ref="A1:BU12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -627,6 +627,8 @@
     <col width="14" customWidth="1" min="69" max="69"/>
     <col width="14" customWidth="1" min="70" max="70"/>
     <col width="14" customWidth="1" min="71" max="71"/>
+    <col width="14" customWidth="1" min="72" max="72"/>
+    <col width="14" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -845,6 +847,12 @@
         </is>
       </c>
       <c r="BS1" s="3" t="n"/>
+      <c r="BT1" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="BU1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1198,6 +1206,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BT2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BU2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1485,6 +1503,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BT3" s="7" t="n">
+        <v>24700</v>
+      </c>
+      <c r="BU3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1772,6 +1798,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BT4" s="9" t="n">
+        <v>38850</v>
+      </c>
+      <c r="BU4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1989,6 +2023,12 @@
       <c r="BS5" s="7" t="n">
         <v>34200</v>
       </c>
+      <c r="BT5" s="7" t="n">
+        <v>34450</v>
+      </c>
+      <c r="BU5" s="7" t="n">
+        <v>33900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2276,6 +2316,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BT6" s="9" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="BU6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2563,6 +2611,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BT7" s="7" t="n">
+        <v>28750</v>
+      </c>
+      <c r="BU7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2920,6 +2976,16 @@
           <t>2026-05-21</t>
         </is>
       </c>
+      <c r="BT8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="BU8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3137,6 +3203,12 @@
       <c r="BS9" s="13" t="n">
         <v>42350</v>
       </c>
+      <c r="BT9" s="13" t="n">
+        <v>38650</v>
+      </c>
+      <c r="BU9" s="13" t="n">
+        <v>42000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3354,6 +3426,12 @@
       <c r="BS10" s="16" t="n">
         <v>-672.04</v>
       </c>
+      <c r="BT10" s="16" t="n">
+        <v>-960.14</v>
+      </c>
+      <c r="BU10" s="16" t="n">
+        <v>-703.12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3571,6 +3649,12 @@
       <c r="BS11" s="13" t="n">
         <v>46350</v>
       </c>
+      <c r="BT11" s="13" t="n">
+        <v>41700</v>
+      </c>
+      <c r="BU11" s="13" t="n">
+        <v>45700</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3787,6 +3871,12 @@
       </c>
       <c r="BS12" s="15" t="n">
         <v>603.78</v>
+      </c>
+      <c r="BT12" s="16" t="n">
+        <v>-607.02</v>
+      </c>
+      <c r="BU12" s="15" t="n">
+        <v>275.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-05-28
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BU12"/>
+  <dimension ref="A1:BW12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -629,6 +629,8 @@
     <col width="14" customWidth="1" min="71" max="71"/>
     <col width="14" customWidth="1" min="72" max="72"/>
     <col width="14" customWidth="1" min="73" max="73"/>
+    <col width="14" customWidth="1" min="74" max="74"/>
+    <col width="14" customWidth="1" min="75" max="75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -853,6 +855,12 @@
         </is>
       </c>
       <c r="BU1" s="3" t="n"/>
+      <c r="BV1" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="BW1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1216,6 +1224,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BV2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BW2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1511,6 +1529,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BV3" s="7" t="n">
+        <v>25250</v>
+      </c>
+      <c r="BW3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1806,6 +1832,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BV4" s="9" t="n">
+        <v>38350</v>
+      </c>
+      <c r="BW4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2029,6 +2063,12 @@
       <c r="BU5" s="7" t="n">
         <v>33900</v>
       </c>
+      <c r="BV5" s="7" t="n">
+        <v>34900</v>
+      </c>
+      <c r="BW5" s="7" t="n">
+        <v>34900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2324,6 +2364,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BV6" s="9" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="BW6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2619,6 +2667,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BV7" s="7" t="n">
+        <v>29700</v>
+      </c>
+      <c r="BW7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2986,6 +3042,16 @@
           <t>2026-05-25</t>
         </is>
       </c>
+      <c r="BV8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="BW8" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3209,6 +3275,12 @@
       <c r="BU9" s="13" t="n">
         <v>42000</v>
       </c>
+      <c r="BV9" s="13" t="n">
+        <v>39550</v>
+      </c>
+      <c r="BW9" s="13" t="n">
+        <v>43000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3432,6 +3504,12 @@
       <c r="BU10" s="16" t="n">
         <v>-703.12</v>
       </c>
+      <c r="BV10" s="16" t="n">
+        <v>-618.1799999999999</v>
+      </c>
+      <c r="BW10" s="16" t="n">
+        <v>-419.08</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3655,6 +3733,12 @@
       <c r="BU11" s="13" t="n">
         <v>45700</v>
       </c>
+      <c r="BV11" s="13" t="n">
+        <v>42700</v>
+      </c>
+      <c r="BW11" s="13" t="n">
+        <v>47800</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3877,6 +3961,12 @@
       </c>
       <c r="BU12" s="15" t="n">
         <v>275.25</v>
+      </c>
+      <c r="BV12" s="16" t="n">
+        <v>-169.52</v>
+      </c>
+      <c r="BW12" s="15" t="n">
+        <v>1653.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-06-08
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BW12"/>
+  <dimension ref="A1:BY12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -631,6 +631,8 @@
     <col width="14" customWidth="1" min="73" max="73"/>
     <col width="14" customWidth="1" min="74" max="74"/>
     <col width="14" customWidth="1" min="75" max="75"/>
+    <col width="14" customWidth="1" min="76" max="76"/>
+    <col width="14" customWidth="1" min="77" max="77"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -861,6 +863,12 @@
         </is>
       </c>
       <c r="BW1" s="3" t="n"/>
+      <c r="BX1" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="BY1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1234,6 +1242,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BX2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="BY2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1537,6 +1555,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BX3" s="7" t="n">
+        <v>24400</v>
+      </c>
+      <c r="BY3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1840,6 +1866,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BX4" s="9" t="n">
+        <v>37750</v>
+      </c>
+      <c r="BY4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2069,6 +2103,12 @@
       <c r="BW5" s="7" t="n">
         <v>34900</v>
       </c>
+      <c r="BX5" s="7" t="n">
+        <v>34750</v>
+      </c>
+      <c r="BY5" s="7" t="n">
+        <v>34800</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2372,6 +2412,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BX6" s="9" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="BY6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2675,6 +2723,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BX7" s="7" t="n">
+        <v>28800</v>
+      </c>
+      <c r="BY7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3052,6 +3108,16 @@
           <t>2026-05-28</t>
         </is>
       </c>
+      <c r="BX8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="BY8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3281,6 +3347,12 @@
       <c r="BW9" s="13" t="n">
         <v>43000</v>
       </c>
+      <c r="BX9" s="13" t="n">
+        <v>38950</v>
+      </c>
+      <c r="BY9" s="13" t="n">
+        <v>42850</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3510,6 +3582,12 @@
       <c r="BW10" s="16" t="n">
         <v>-419.08</v>
       </c>
+      <c r="BX10" s="16" t="n">
+        <v>-313.11</v>
+      </c>
+      <c r="BY10" s="16" t="n">
+        <v>-48.34</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3739,6 +3817,12 @@
       <c r="BW11" s="13" t="n">
         <v>47800</v>
       </c>
+      <c r="BX11" s="13" t="n">
+        <v>41900</v>
+      </c>
+      <c r="BY11" s="13" t="n">
+        <v>47500</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -3967,6 +4051,12 @@
       </c>
       <c r="BW12" s="15" t="n">
         <v>1653.57</v>
+      </c>
+      <c r="BX12" s="16" t="n">
+        <v>-57.22</v>
+      </c>
+      <c r="BY12" s="15" t="n">
+        <v>1878.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-06-15
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BY12"/>
+  <dimension ref="A1:CA12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -633,6 +633,8 @@
     <col width="14" customWidth="1" min="75" max="75"/>
     <col width="14" customWidth="1" min="76" max="76"/>
     <col width="14" customWidth="1" min="77" max="77"/>
+    <col width="14" customWidth="1" min="78" max="78"/>
+    <col width="14" customWidth="1" min="79" max="79"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -869,6 +871,12 @@
         </is>
       </c>
       <c r="BY1" s="3" t="n"/>
+      <c r="BZ1" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="CA1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1252,6 +1260,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="BZ2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CA2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1563,6 +1581,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BZ3" s="7" t="n">
+        <v>24100</v>
+      </c>
+      <c r="CA3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1874,6 +1900,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BZ4" s="9" t="n">
+        <v>37400</v>
+      </c>
+      <c r="CA4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2109,6 +2143,12 @@
       <c r="BY5" s="7" t="n">
         <v>34800</v>
       </c>
+      <c r="BZ5" s="7" t="n">
+        <v>34400</v>
+      </c>
+      <c r="CA5" s="7" t="n">
+        <v>34500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2420,6 +2460,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BZ6" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="CA6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2731,6 +2779,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="BZ7" s="7" t="n">
+        <v>28650</v>
+      </c>
+      <c r="CA7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3118,6 +3174,16 @@
           <t>2026-06-08</t>
         </is>
       </c>
+      <c r="BZ8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="CA8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3353,6 +3419,12 @@
       <c r="BY9" s="13" t="n">
         <v>42850</v>
       </c>
+      <c r="BZ9" s="13" t="n">
+        <v>38800</v>
+      </c>
+      <c r="CA9" s="13" t="n">
+        <v>42500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3588,6 +3660,12 @@
       <c r="BY10" s="16" t="n">
         <v>-48.34</v>
       </c>
+      <c r="BZ10" s="16" t="n">
+        <v>-117.52</v>
+      </c>
+      <c r="CA10" s="16" t="n">
+        <v>-61.51</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3823,6 +3901,12 @@
       <c r="BY11" s="13" t="n">
         <v>47500</v>
       </c>
+      <c r="BZ11" s="13" t="n">
+        <v>41500</v>
+      </c>
+      <c r="CA11" s="13" t="n">
+        <v>46900</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4057,6 +4141,12 @@
       </c>
       <c r="BY12" s="15" t="n">
         <v>1878.47</v>
+      </c>
+      <c r="BZ12" s="16" t="n">
+        <v>-108.86</v>
+      </c>
+      <c r="CA12" s="15" t="n">
+        <v>1618</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-06-22
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA12"/>
+  <dimension ref="A1:CC12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,8 @@
     <col width="14" customWidth="1" min="77" max="77"/>
     <col width="14" customWidth="1" min="78" max="78"/>
     <col width="14" customWidth="1" min="79" max="79"/>
+    <col width="14" customWidth="1" min="80" max="80"/>
+    <col width="14" customWidth="1" min="81" max="81"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -877,6 +879,12 @@
         </is>
       </c>
       <c r="CA1" s="3" t="n"/>
+      <c r="CB1" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="CC1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1270,6 +1278,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CB2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CC2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1589,6 +1607,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CB3" s="7" t="n">
+        <v>24100</v>
+      </c>
+      <c r="CC3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1908,6 +1934,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CB4" s="9" t="n">
+        <v>37200</v>
+      </c>
+      <c r="CC4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2149,6 +2183,12 @@
       <c r="CA5" s="7" t="n">
         <v>34500</v>
       </c>
+      <c r="CB5" s="7" t="n">
+        <v>34400</v>
+      </c>
+      <c r="CC5" s="7" t="n">
+        <v>34500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2468,6 +2508,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CB6" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="CC6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2787,6 +2835,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CB7" s="7" t="n">
+        <v>28550</v>
+      </c>
+      <c r="CC7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3184,6 +3240,16 @@
           <t>2026-06-15</t>
         </is>
       </c>
+      <c r="CB8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="CC8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3425,6 +3491,12 @@
       <c r="CA9" s="13" t="n">
         <v>42500</v>
       </c>
+      <c r="CB9" s="13" t="n">
+        <v>38850</v>
+      </c>
+      <c r="CC9" s="13" t="n">
+        <v>42350</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3666,6 +3738,12 @@
       <c r="CA10" s="16" t="n">
         <v>-61.51</v>
       </c>
+      <c r="CB10" s="16" t="n">
+        <v>-44.08</v>
+      </c>
+      <c r="CC10" s="16" t="n">
+        <v>-199.98</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3907,6 +3985,12 @@
       <c r="CA11" s="13" t="n">
         <v>46900</v>
       </c>
+      <c r="CB11" s="13" t="n">
+        <v>41900</v>
+      </c>
+      <c r="CC11" s="13" t="n">
+        <v>46500</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4147,6 +4231,12 @@
       </c>
       <c r="CA12" s="15" t="n">
         <v>1618</v>
+      </c>
+      <c r="CB12" s="15" t="n">
+        <v>314.77</v>
+      </c>
+      <c r="CC12" s="15" t="n">
+        <v>1229.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-06-30
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CC12"/>
+  <dimension ref="A1:CE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,8 @@
     <col width="14" customWidth="1" min="79" max="79"/>
     <col width="14" customWidth="1" min="80" max="80"/>
     <col width="14" customWidth="1" min="81" max="81"/>
+    <col width="14" customWidth="1" min="82" max="82"/>
+    <col width="14" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -885,6 +887,12 @@
         </is>
       </c>
       <c r="CC1" s="3" t="n"/>
+      <c r="CD1" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="CE1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1288,6 +1296,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CD2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CE2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1615,6 +1633,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CD3" s="7" t="n">
+        <v>24150</v>
+      </c>
+      <c r="CE3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1942,6 +1968,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CD4" s="9" t="n">
+        <v>37150</v>
+      </c>
+      <c r="CE4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2189,6 +2223,12 @@
       <c r="CC5" s="7" t="n">
         <v>34500</v>
       </c>
+      <c r="CD5" s="7" t="n">
+        <v>34300</v>
+      </c>
+      <c r="CE5" s="7" t="n">
+        <v>34900</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2516,6 +2556,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CD6" s="9" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="CE6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2843,6 +2891,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CD7" s="7" t="n">
+        <v>28250</v>
+      </c>
+      <c r="CE7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3250,6 +3306,16 @@
           <t>2026-06-22</t>
         </is>
       </c>
+      <c r="CD8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="CE8" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3497,6 +3563,12 @@
       <c r="CC9" s="13" t="n">
         <v>42350</v>
       </c>
+      <c r="CD9" s="13" t="n">
+        <v>39100</v>
+      </c>
+      <c r="CE9" s="13" t="n">
+        <v>42700</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3744,6 +3816,12 @@
       <c r="CC10" s="16" t="n">
         <v>-199.98</v>
       </c>
+      <c r="CD10" s="15" t="n">
+        <v>213.13</v>
+      </c>
+      <c r="CE10" s="16" t="n">
+        <v>-78.78</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3991,6 +4069,12 @@
       <c r="CC11" s="13" t="n">
         <v>46500</v>
       </c>
+      <c r="CD11" s="13" t="n">
+        <v>41600</v>
+      </c>
+      <c r="CE11" s="13" t="n">
+        <v>46700</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4237,6 +4321,12 @@
       </c>
       <c r="CC12" s="15" t="n">
         <v>1229.63</v>
+      </c>
+      <c r="CD12" s="15" t="n">
+        <v>22.04</v>
+      </c>
+      <c r="CE12" s="15" t="n">
+        <v>1198.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-07-08
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CE12"/>
+  <dimension ref="A1:CG12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -639,6 +639,8 @@
     <col width="14" customWidth="1" min="81" max="81"/>
     <col width="14" customWidth="1" min="82" max="82"/>
     <col width="14" customWidth="1" min="83" max="83"/>
+    <col width="14" customWidth="1" min="84" max="84"/>
+    <col width="14" customWidth="1" min="85" max="85"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -893,6 +895,12 @@
         </is>
       </c>
       <c r="CE1" s="3" t="n"/>
+      <c r="CF1" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="CG1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1306,6 +1314,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CF2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CG2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1641,6 +1659,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CF3" s="7" t="n">
+        <v>23100</v>
+      </c>
+      <c r="CG3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1976,6 +2002,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CF4" s="9" t="n">
+        <v>37550</v>
+      </c>
+      <c r="CG4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2229,6 +2263,12 @@
       <c r="CE5" s="7" t="n">
         <v>34900</v>
       </c>
+      <c r="CF5" s="7" t="n">
+        <v>34000</v>
+      </c>
+      <c r="CG5" s="7" t="n">
+        <v>33500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2564,6 +2604,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CF6" s="9" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="CG6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2899,6 +2947,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CF7" s="7" t="n">
+        <v>27100</v>
+      </c>
+      <c r="CG7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3316,6 +3372,16 @@
           <t>2026-06-30</t>
         </is>
       </c>
+      <c r="CF8" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="CG8" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3569,6 +3635,12 @@
       <c r="CE9" s="13" t="n">
         <v>42700</v>
       </c>
+      <c r="CF9" s="13" t="n">
+        <v>38000</v>
+      </c>
+      <c r="CG9" s="13" t="n">
+        <v>41600</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3822,6 +3894,12 @@
       <c r="CE10" s="16" t="n">
         <v>-78.78</v>
       </c>
+      <c r="CF10" s="15" t="n">
+        <v>140.93</v>
+      </c>
+      <c r="CG10" s="15" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4075,6 +4153,12 @@
       <c r="CE11" s="13" t="n">
         <v>46700</v>
       </c>
+      <c r="CF11" s="13" t="n">
+        <v>40200</v>
+      </c>
+      <c r="CG11" s="13" t="n">
+        <v>44350</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4327,6 +4411,12 @@
       </c>
       <c r="CE12" s="15" t="n">
         <v>1198.99</v>
+      </c>
+      <c r="CF12" s="16" t="n">
+        <v>-341.95</v>
+      </c>
+      <c r="CG12" s="15" t="n">
+        <v>59.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update costing output for 2026-07-14
</commit_message>
<xml_diff>
--- a/output/change_log.xlsx
+++ b/output/change_log.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CG12"/>
+  <dimension ref="A1:CI12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,8 @@
     <col width="14" customWidth="1" min="83" max="83"/>
     <col width="14" customWidth="1" min="84" max="84"/>
     <col width="14" customWidth="1" min="85" max="85"/>
+    <col width="14" customWidth="1" min="86" max="86"/>
+    <col width="14" customWidth="1" min="87" max="87"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -901,6 +903,12 @@
         </is>
       </c>
       <c r="CG1" s="3" t="n"/>
+      <c r="CH1" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="CI1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -1324,6 +1332,16 @@
           <t>NCR</t>
         </is>
       </c>
+      <c r="CH2" s="4" t="inlineStr">
+        <is>
+          <t>Raipur</t>
+        </is>
+      </c>
+      <c r="CI2" s="5" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1667,6 +1685,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CH3" s="7" t="n">
+        <v>22950</v>
+      </c>
+      <c r="CI3" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2010,6 +2036,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CH4" s="9" t="n">
+        <v>38000</v>
+      </c>
+      <c r="CI4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2269,6 +2303,12 @@
       <c r="CG5" s="7" t="n">
         <v>33500</v>
       </c>
+      <c r="CH5" s="7" t="n">
+        <v>34000</v>
+      </c>
+      <c r="CI5" s="7" t="n">
+        <v>33300</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2612,6 +2652,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CH6" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="CI6" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2955,6 +3003,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="CH7" s="7" t="n">
+        <v>26900</v>
+      </c>
+      <c r="CI7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3382,6 +3438,16 @@
           <t>2026-07-08</t>
         </is>
       </c>
+      <c r="CH8" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="CI8" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3641,6 +3707,12 @@
       <c r="CG9" s="13" t="n">
         <v>41600</v>
       </c>
+      <c r="CH9" s="13" t="n">
+        <v>37450</v>
+      </c>
+      <c r="CI9" s="13" t="n">
+        <v>41300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -3900,6 +3972,12 @@
       <c r="CG10" s="15" t="n">
         <v>22.59</v>
       </c>
+      <c r="CH10" s="16" t="n">
+        <v>-302.61</v>
+      </c>
+      <c r="CI10" s="16" t="n">
+        <v>-145.94</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4159,6 +4237,12 @@
       <c r="CG11" s="13" t="n">
         <v>44350</v>
       </c>
+      <c r="CH11" s="13" t="n">
+        <v>39300</v>
+      </c>
+      <c r="CI11" s="13" t="n">
+        <v>43600</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
@@ -4417,6 +4501,12 @@
       </c>
       <c r="CG12" s="15" t="n">
         <v>59.97</v>
+      </c>
+      <c r="CH12" s="16" t="n">
+        <v>-1134.63</v>
+      </c>
+      <c r="CI12" s="16" t="n">
+        <v>-557.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>